<commit_message>
be5f49b - 16.1 장비 작업
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/DropTable.xlsx
+++ b/JsonConverter/ExcelFiles/DropTable.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
   <si>
     <t xml:space="preserve">드랍테이블 고유 ID</t>
   </si>
@@ -56,6 +56,228 @@
   </si>
   <si>
     <t xml:space="preserve">DropTable_0001</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Gold_0001,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">Fuel_0002,Supplies_0003,TradingGoods_0004</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50,50,50,5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1,1,1,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">10,2,2,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DropTable_0002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50,2,2,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DropTable_0003</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Gold_0001,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">Fuel_0002,Supplies_0003,TradingGoods_0004,TradingGoods_0005</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50,50,50,5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">0,50</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1,1,1,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">1,1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">100,2,2,2,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DropTable_0004</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Gold_0001,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">Fuel_0002,Supplies_0003,TradingGoods_0004,TradingGoods_0005,TradingGoods_0006</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50,50,50,5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="&quot;맑은 고딕&quot;"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">0,50,50</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1,1,1,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">1,1,1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">200,2,2,2,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DropTable_0005</t>
   </si>
   <si>
     <r>
@@ -88,7 +310,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">100,100,100,</t>
+      <t xml:space="preserve">50,50,50,5</t>
     </r>
     <r>
       <rPr>
@@ -98,52 +320,14 @@
         <family val="0"/>
         <charset val="129"/>
       </rPr>
-      <t xml:space="preserve">100,100,100,100</t>
+      <t xml:space="preserve">0,50,50,50</t>
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1,1,1,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">1,1,1,1</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100,100,100,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">100,100,100,100</t>
-    </r>
+    <t xml:space="preserve">1,1,1,1,1,1,1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">500,2,2,2,2</t>
   </si>
 </sst>
 </file>
@@ -326,12 +510,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -681,11 +865,21 @@
       <c r="L4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="10"/>
+      <c r="A5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>17</v>
+      </c>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
@@ -695,11 +889,21 @@
       <c r="L5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
+      <c r="A6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>22</v>
+      </c>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
@@ -709,11 +913,21 @@
       <c r="L6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
+      <c r="A7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="F7" s="11"/>
       <c r="G7" s="11"/>
       <c r="H7" s="11"/>
@@ -723,11 +937,21 @@
       <c r="L7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
+      <c r="A8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>32</v>
+      </c>
       <c r="F8" s="11"/>
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>

</xml_diff>